<commit_message>
Rank Doctors and Employees separately in descending order by attendance
</commit_message>
<xml_diff>
--- a/Vasus_Attendance_August_2026.xlsx
+++ b/Vasus_Attendance_August_2026.xlsx
@@ -359,12 +359,6 @@
     <xf numFmtId="0" fontId="8" fillId="9" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="12" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -394,6 +388,12 @@
     </xf>
     <xf numFmtId="0" fontId="6" fillId="20" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="11" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -823,14 +823,14 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>VASUS ATTENDANCE TRACKER — AUGUST 2026</t>
+          <t>VASUS ATTENDANCE TRACKER — AUGUST 2026 (RANKED IN DESCENDING ORDER)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Status Codes:  [P] Present (Green)  |  [CL] Casual Leave (Teal)  |  [L] Leave (Red)  |  [WO] Week Off (Purple)  |  [HO] Holiday (Mint)  |  [CF] Comp Off (Pink)  |  [-] Blank</t>
+          <t>Doctors &amp; Employees ranked in descending order separately  |  [P] Present (Green)  [CL] Casual Leave (Teal)  [L] Leave (Red)  [WO] Week Off (Purple)  [CF] Comp Off (Pink)</t>
         </is>
       </c>
     </row>
@@ -1073,7 +1073,7 @@
     <row r="5" ht="32" customHeight="1">
       <c r="A5" s="12" t="inlineStr">
         <is>
-          <t>DR BINDU
+          <t>DR PRANAY
 Doctor</t>
         </is>
       </c>
@@ -1082,9 +1082,9 @@
           <t>P</t>
         </is>
       </c>
-      <c r="C5" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
         </is>
       </c>
       <c r="D5" s="13" t="inlineStr">
@@ -1112,29 +1112,29 @@
           <t>P</t>
         </is>
       </c>
-      <c r="I5" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="J5" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="K5" s="15" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="L5" s="16" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="M5" s="16" t="inlineStr">
-        <is>
-          <t>L</t>
+      <c r="I5" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="J5" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="K5" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="L5" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="M5" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
         </is>
       </c>
       <c r="N5" s="13" t="inlineStr">
@@ -1147,14 +1147,14 @@
           <t>P</t>
         </is>
       </c>
-      <c r="P5" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="Q5" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
+      <c r="P5" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="Q5" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
         </is>
       </c>
       <c r="R5" s="13" t="inlineStr">
@@ -1182,14 +1182,14 @@
           <t>P</t>
         </is>
       </c>
-      <c r="W5" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="X5" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
+      <c r="W5" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="X5" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
         </is>
       </c>
       <c r="Y5" s="13" t="inlineStr">
@@ -1217,56 +1217,56 @@
           <t>P</t>
         </is>
       </c>
-      <c r="AD5" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AE5" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="AF5" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG5" s="18">
+      <c r="AD5" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="AE5" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AF5" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG5" s="16">
         <f>COUNTIF(B5:AF5, "P")</f>
         <v/>
       </c>
-      <c r="AH5" s="19">
+      <c r="AH5" s="17">
         <f>COUNTIF(B5:AF5, "CL")</f>
         <v/>
       </c>
-      <c r="AI5" s="20">
+      <c r="AI5" s="18">
         <f>COUNTIF(B5:AF5, "L")</f>
         <v/>
       </c>
-      <c r="AJ5" s="21">
+      <c r="AJ5" s="19">
         <f>COUNTIF(B5:AF5, "WO")</f>
         <v/>
       </c>
-      <c r="AK5" s="22">
+      <c r="AK5" s="20">
         <f>COUNTIF(B5:AF5, "HO")</f>
         <v/>
       </c>
-      <c r="AL5" s="23">
+      <c r="AL5" s="21">
         <f>COUNTIF(B5:AF5, "CF")</f>
         <v/>
       </c>
-      <c r="AM5" s="24">
+      <c r="AM5" s="22">
         <f>AG5+AH5+AI5+AL5</f>
         <v/>
       </c>
-      <c r="AN5" s="25">
+      <c r="AN5" s="23">
         <f>IF(AM5&gt;0, AG5/AM5, 0)</f>
         <v/>
       </c>
     </row>
     <row r="6" ht="32" customHeight="1">
-      <c r="A6" s="26" t="inlineStr">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>DR CHINJU
 Doctor</t>
@@ -1422,40 +1422,40 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="AF6" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG6" s="18">
+      <c r="AF6" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG6" s="16">
         <f>COUNTIF(B6:AF6, "P")</f>
         <v/>
       </c>
-      <c r="AH6" s="19">
+      <c r="AH6" s="17">
         <f>COUNTIF(B6:AF6, "CL")</f>
         <v/>
       </c>
-      <c r="AI6" s="20">
+      <c r="AI6" s="18">
         <f>COUNTIF(B6:AF6, "L")</f>
         <v/>
       </c>
-      <c r="AJ6" s="21">
+      <c r="AJ6" s="19">
         <f>COUNTIF(B6:AF6, "WO")</f>
         <v/>
       </c>
-      <c r="AK6" s="22">
+      <c r="AK6" s="20">
         <f>COUNTIF(B6:AF6, "HO")</f>
         <v/>
       </c>
-      <c r="AL6" s="23">
+      <c r="AL6" s="21">
         <f>COUNTIF(B6:AF6, "CF")</f>
         <v/>
       </c>
-      <c r="AM6" s="24">
+      <c r="AM6" s="22">
         <f>AG6+AH6+AI6+AL6</f>
         <v/>
       </c>
-      <c r="AN6" s="25">
+      <c r="AN6" s="23">
         <f>IF(AM6&gt;0, AG6/AM6, 0)</f>
         <v/>
       </c>
@@ -1463,7 +1463,7 @@
     <row r="7" ht="32" customHeight="1">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>DR PRANAY
+          <t>DR SUNITHA
 Doctor</t>
         </is>
       </c>
@@ -1472,9 +1472,9 @@
           <t>P</t>
         </is>
       </c>
-      <c r="C7" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="C7" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
         </is>
       </c>
       <c r="D7" s="13" t="inlineStr">
@@ -1502,14 +1502,14 @@
           <t>P</t>
         </is>
       </c>
-      <c r="I7" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="J7" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="I7" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="J7" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
         </is>
       </c>
       <c r="K7" s="13" t="inlineStr">
@@ -1537,14 +1537,14 @@
           <t>P</t>
         </is>
       </c>
-      <c r="P7" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="Q7" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="P7" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Q7" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
         </is>
       </c>
       <c r="R7" s="13" t="inlineStr">
@@ -1572,14 +1572,14 @@
           <t>P</t>
         </is>
       </c>
-      <c r="W7" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="X7" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="W7" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="X7" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
         </is>
       </c>
       <c r="Y7" s="13" t="inlineStr">
@@ -1607,58 +1607,58 @@
           <t>P</t>
         </is>
       </c>
-      <c r="AD7" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="AE7" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AF7" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG7" s="18">
+      <c r="AD7" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AE7" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="AF7" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG7" s="16">
         <f>COUNTIF(B7:AF7, "P")</f>
         <v/>
       </c>
-      <c r="AH7" s="19">
+      <c r="AH7" s="17">
         <f>COUNTIF(B7:AF7, "CL")</f>
         <v/>
       </c>
-      <c r="AI7" s="20">
+      <c r="AI7" s="18">
         <f>COUNTIF(B7:AF7, "L")</f>
         <v/>
       </c>
-      <c r="AJ7" s="21">
+      <c r="AJ7" s="19">
         <f>COUNTIF(B7:AF7, "WO")</f>
         <v/>
       </c>
-      <c r="AK7" s="22">
+      <c r="AK7" s="20">
         <f>COUNTIF(B7:AF7, "HO")</f>
         <v/>
       </c>
-      <c r="AL7" s="23">
+      <c r="AL7" s="21">
         <f>COUNTIF(B7:AF7, "CF")</f>
         <v/>
       </c>
-      <c r="AM7" s="24">
+      <c r="AM7" s="22">
         <f>AG7+AH7+AI7+AL7</f>
         <v/>
       </c>
-      <c r="AN7" s="25">
+      <c r="AN7" s="23">
         <f>IF(AM7&gt;0, AG7/AM7, 0)</f>
         <v/>
       </c>
     </row>
     <row r="8" ht="32" customHeight="1">
-      <c r="A8" s="26" t="inlineStr">
-        <is>
-          <t>DR SUNITHA
+      <c r="A8" s="24" t="inlineStr">
+        <is>
+          <t>DR BINDU
 Doctor</t>
         </is>
       </c>
@@ -1707,19 +1707,19 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="K8" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="L8" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="M8" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="K8" s="25" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="L8" s="26" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="M8" s="26" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="N8" s="13" t="inlineStr">
@@ -1812,40 +1812,40 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="AF8" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG8" s="18">
+      <c r="AF8" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG8" s="16">
         <f>COUNTIF(B8:AF8, "P")</f>
         <v/>
       </c>
-      <c r="AH8" s="19">
+      <c r="AH8" s="17">
         <f>COUNTIF(B8:AF8, "CL")</f>
         <v/>
       </c>
-      <c r="AI8" s="20">
+      <c r="AI8" s="18">
         <f>COUNTIF(B8:AF8, "L")</f>
         <v/>
       </c>
-      <c r="AJ8" s="21">
+      <c r="AJ8" s="19">
         <f>COUNTIF(B8:AF8, "WO")</f>
         <v/>
       </c>
-      <c r="AK8" s="22">
+      <c r="AK8" s="20">
         <f>COUNTIF(B8:AF8, "HO")</f>
         <v/>
       </c>
-      <c r="AL8" s="23">
+      <c r="AL8" s="21">
         <f>COUNTIF(B8:AF8, "CF")</f>
         <v/>
       </c>
-      <c r="AM8" s="24">
+      <c r="AM8" s="22">
         <f>AG8+AH8+AI8+AL8</f>
         <v/>
       </c>
-      <c r="AN8" s="25">
+      <c r="AN8" s="23">
         <f>IF(AM8&gt;0, AG8/AM8, 0)</f>
         <v/>
       </c>
@@ -1937,32 +1937,32 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="R9" s="15" t="inlineStr">
+      <c r="R9" s="25" t="inlineStr">
         <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="S9" s="16" t="inlineStr">
+      <c r="S9" s="26" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="T9" s="16" t="inlineStr">
+      <c r="T9" s="26" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="U9" s="16" t="inlineStr">
+      <c r="U9" s="26" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="V9" s="16" t="inlineStr">
+      <c r="V9" s="26" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="W9" s="16" t="inlineStr">
+      <c r="W9" s="26" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -1972,32 +1972,32 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="Y9" s="16" t="inlineStr">
+      <c r="Y9" s="26" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="Z9" s="16" t="inlineStr">
+      <c r="Z9" s="26" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="AA9" s="16" t="inlineStr">
+      <c r="AA9" s="26" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="AB9" s="16" t="inlineStr">
+      <c r="AB9" s="26" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="AC9" s="16" t="inlineStr">
+      <c r="AC9" s="26" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="AD9" s="16" t="inlineStr">
+      <c r="AD9" s="26" t="inlineStr">
         <is>
           <t>L</t>
         </is>
@@ -2007,48 +2007,48 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="AF9" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG9" s="18">
+      <c r="AF9" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG9" s="16">
         <f>COUNTIF(B9:AF9, "P")</f>
         <v/>
       </c>
-      <c r="AH9" s="19">
+      <c r="AH9" s="17">
         <f>COUNTIF(B9:AF9, "CL")</f>
         <v/>
       </c>
-      <c r="AI9" s="20">
+      <c r="AI9" s="18">
         <f>COUNTIF(B9:AF9, "L")</f>
         <v/>
       </c>
-      <c r="AJ9" s="21">
+      <c r="AJ9" s="19">
         <f>COUNTIF(B9:AF9, "WO")</f>
         <v/>
       </c>
-      <c r="AK9" s="22">
+      <c r="AK9" s="20">
         <f>COUNTIF(B9:AF9, "HO")</f>
         <v/>
       </c>
-      <c r="AL9" s="23">
+      <c r="AL9" s="21">
         <f>COUNTIF(B9:AF9, "CF")</f>
         <v/>
       </c>
-      <c r="AM9" s="24">
+      <c r="AM9" s="22">
         <f>AG9+AH9+AI9+AL9</f>
         <v/>
       </c>
-      <c r="AN9" s="25">
+      <c r="AN9" s="23">
         <f>IF(AM9&gt;0, AG9/AM9, 0)</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="32" customHeight="1">
-      <c r="A10" s="26" t="inlineStr">
-        <is>
-          <t>CHANIKYA
+      <c r="A10" s="24" t="inlineStr">
+        <is>
+          <t>NEELIMA
 Employee</t>
         </is>
       </c>
@@ -2067,9 +2067,9 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E10" s="15" t="inlineStr">
-        <is>
-          <t>CL</t>
+      <c r="E10" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
         </is>
       </c>
       <c r="F10" s="13" t="inlineStr">
@@ -2122,14 +2122,14 @@
           <t>P</t>
         </is>
       </c>
-      <c r="P10" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q10" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
+      <c r="P10" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Q10" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
         </is>
       </c>
       <c r="R10" s="13" t="inlineStr">
@@ -2162,9 +2162,9 @@
           <t>P</t>
         </is>
       </c>
-      <c r="X10" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="X10" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
         </is>
       </c>
       <c r="Y10" s="13" t="inlineStr">
@@ -2202,40 +2202,40 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="AF10" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG10" s="18">
+      <c r="AF10" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG10" s="16">
         <f>COUNTIF(B10:AF10, "P")</f>
         <v/>
       </c>
-      <c r="AH10" s="19">
+      <c r="AH10" s="17">
         <f>COUNTIF(B10:AF10, "CL")</f>
         <v/>
       </c>
-      <c r="AI10" s="20">
+      <c r="AI10" s="18">
         <f>COUNTIF(B10:AF10, "L")</f>
         <v/>
       </c>
-      <c r="AJ10" s="21">
+      <c r="AJ10" s="19">
         <f>COUNTIF(B10:AF10, "WO")</f>
         <v/>
       </c>
-      <c r="AK10" s="22">
+      <c r="AK10" s="20">
         <f>COUNTIF(B10:AF10, "HO")</f>
         <v/>
       </c>
-      <c r="AL10" s="23">
+      <c r="AL10" s="21">
         <f>COUNTIF(B10:AF10, "CF")</f>
         <v/>
       </c>
-      <c r="AM10" s="24">
+      <c r="AM10" s="22">
         <f>AG10+AH10+AI10+AL10</f>
         <v/>
       </c>
-      <c r="AN10" s="25">
+      <c r="AN10" s="23">
         <f>IF(AM10&gt;0, AG10/AM10, 0)</f>
         <v/>
       </c>
@@ -2243,7 +2243,7 @@
     <row r="11" ht="32" customHeight="1">
       <c r="A11" s="12" t="inlineStr">
         <is>
-          <t>Ch Praveen Kumar
+          <t>RAMESH
 Employee</t>
         </is>
       </c>
@@ -2252,9 +2252,9 @@
           <t>P</t>
         </is>
       </c>
-      <c r="C11" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="C11" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
         </is>
       </c>
       <c r="D11" s="13" t="inlineStr">
@@ -2277,14 +2277,14 @@
           <t>P</t>
         </is>
       </c>
-      <c r="H11" s="15" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="I11" s="27" t="inlineStr">
-        <is>
-          <t>CF</t>
+      <c r="H11" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="I11" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
         </is>
       </c>
       <c r="J11" s="14" t="inlineStr">
@@ -2317,9 +2317,9 @@
           <t>P</t>
         </is>
       </c>
-      <c r="P11" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="P11" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="Q11" s="14" t="inlineStr">
@@ -2397,48 +2397,48 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="AF11" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG11" s="18">
+      <c r="AF11" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG11" s="16">
         <f>COUNTIF(B11:AF11, "P")</f>
         <v/>
       </c>
-      <c r="AH11" s="19">
+      <c r="AH11" s="17">
         <f>COUNTIF(B11:AF11, "CL")</f>
         <v/>
       </c>
-      <c r="AI11" s="20">
+      <c r="AI11" s="18">
         <f>COUNTIF(B11:AF11, "L")</f>
         <v/>
       </c>
-      <c r="AJ11" s="21">
+      <c r="AJ11" s="19">
         <f>COUNTIF(B11:AF11, "WO")</f>
         <v/>
       </c>
-      <c r="AK11" s="22">
+      <c r="AK11" s="20">
         <f>COUNTIF(B11:AF11, "HO")</f>
         <v/>
       </c>
-      <c r="AL11" s="23">
+      <c r="AL11" s="21">
         <f>COUNTIF(B11:AF11, "CF")</f>
         <v/>
       </c>
-      <c r="AM11" s="24">
+      <c r="AM11" s="22">
         <f>AG11+AH11+AI11+AL11</f>
         <v/>
       </c>
-      <c r="AN11" s="25">
+      <c r="AN11" s="23">
         <f>IF(AM11&gt;0, AG11/AM11, 0)</f>
         <v/>
       </c>
     </row>
     <row r="12" ht="32" customHeight="1">
-      <c r="A12" s="26" t="inlineStr">
-        <is>
-          <t>KAVITHA
+      <c r="A12" s="24" t="inlineStr">
+        <is>
+          <t>SAI KUMAR
 Employee</t>
         </is>
       </c>
@@ -2482,9 +2482,9 @@
           <t>P</t>
         </is>
       </c>
-      <c r="J12" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
+      <c r="J12" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
         </is>
       </c>
       <c r="K12" s="13" t="inlineStr">
@@ -2502,86 +2502,86 @@
           <t>P</t>
         </is>
       </c>
-      <c r="N12" s="15" t="inlineStr">
+      <c r="N12" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="O12" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="P12" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Q12" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="R12" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="S12" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="T12" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="U12" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="V12" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="W12" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="X12" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="Y12" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Z12" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AA12" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AB12" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AC12" s="25" t="inlineStr">
         <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="O12" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="P12" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="Q12" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="R12" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="S12" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="T12" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="U12" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="V12" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="W12" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="X12" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="Y12" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="Z12" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AA12" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AB12" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AC12" s="27" t="inlineStr">
-        <is>
-          <t>CF</t>
-        </is>
-      </c>
       <c r="AD12" s="13" t="inlineStr">
         <is>
           <t>P</t>
@@ -2592,40 +2592,40 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="AF12" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG12" s="18">
+      <c r="AF12" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG12" s="16">
         <f>COUNTIF(B12:AF12, "P")</f>
         <v/>
       </c>
-      <c r="AH12" s="19">
+      <c r="AH12" s="17">
         <f>COUNTIF(B12:AF12, "CL")</f>
         <v/>
       </c>
-      <c r="AI12" s="20">
+      <c r="AI12" s="18">
         <f>COUNTIF(B12:AF12, "L")</f>
         <v/>
       </c>
-      <c r="AJ12" s="21">
+      <c r="AJ12" s="19">
         <f>COUNTIF(B12:AF12, "WO")</f>
         <v/>
       </c>
-      <c r="AK12" s="22">
+      <c r="AK12" s="20">
         <f>COUNTIF(B12:AF12, "HO")</f>
         <v/>
       </c>
-      <c r="AL12" s="23">
+      <c r="AL12" s="21">
         <f>COUNTIF(B12:AF12, "CF")</f>
         <v/>
       </c>
-      <c r="AM12" s="24">
+      <c r="AM12" s="22">
         <f>AG12+AH12+AI12+AL12</f>
         <v/>
       </c>
-      <c r="AN12" s="25">
+      <c r="AN12" s="23">
         <f>IF(AM12&gt;0, AG12/AM12, 0)</f>
         <v/>
       </c>
@@ -2633,318 +2633,318 @@
     <row r="13" ht="32" customHeight="1">
       <c r="A13" s="12" t="inlineStr">
         <is>
+          <t>CHANIKYA
+Employee</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C13" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E13" s="25" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="G13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="H13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="I13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="J13" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="K13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="L13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="M13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="N13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="O13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="P13" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q13" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="R13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="S13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="T13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="U13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="V13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="W13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="X13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Y13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Z13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AA13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AB13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AC13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AD13" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AE13" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="AF13" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG13" s="16">
+        <f>COUNTIF(B13:AF13, "P")</f>
+        <v/>
+      </c>
+      <c r="AH13" s="17">
+        <f>COUNTIF(B13:AF13, "CL")</f>
+        <v/>
+      </c>
+      <c r="AI13" s="18">
+        <f>COUNTIF(B13:AF13, "L")</f>
+        <v/>
+      </c>
+      <c r="AJ13" s="19">
+        <f>COUNTIF(B13:AF13, "WO")</f>
+        <v/>
+      </c>
+      <c r="AK13" s="20">
+        <f>COUNTIF(B13:AF13, "HO")</f>
+        <v/>
+      </c>
+      <c r="AL13" s="21">
+        <f>COUNTIF(B13:AF13, "CF")</f>
+        <v/>
+      </c>
+      <c r="AM13" s="22">
+        <f>AG13+AH13+AI13+AL13</f>
+        <v/>
+      </c>
+      <c r="AN13" s="23">
+        <f>IF(AM13&gt;0, AG13/AM13, 0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14" ht="32" customHeight="1">
+      <c r="A14" s="24" t="inlineStr">
+        <is>
           <t>LAXMINARAYANA
 Employee</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="C13" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="D13" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="E13" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="F13" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="G13" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="H13" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="I13" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="J13" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="K13" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="L13" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="M13" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="N13" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="O13" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="P13" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q13" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="R13" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="S13" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="T13" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="U13" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="V13" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="W13" s="15" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C14" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="D14" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E14" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="F14" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="G14" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="H14" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="I14" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="J14" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="K14" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="L14" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="M14" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="N14" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="O14" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="P14" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q14" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="R14" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="S14" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="T14" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="U14" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="V14" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="W14" s="25" t="inlineStr">
         <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="X13" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="Y13" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="Z13" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AA13" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AB13" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AC13" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AD13" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AE13" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="AF13" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG13" s="18">
-        <f>COUNTIF(B13:AF13, "P")</f>
-        <v/>
-      </c>
-      <c r="AH13" s="19">
-        <f>COUNTIF(B13:AF13, "CL")</f>
-        <v/>
-      </c>
-      <c r="AI13" s="20">
-        <f>COUNTIF(B13:AF13, "L")</f>
-        <v/>
-      </c>
-      <c r="AJ13" s="21">
-        <f>COUNTIF(B13:AF13, "WO")</f>
-        <v/>
-      </c>
-      <c r="AK13" s="22">
-        <f>COUNTIF(B13:AF13, "HO")</f>
-        <v/>
-      </c>
-      <c r="AL13" s="23">
-        <f>COUNTIF(B13:AF13, "CF")</f>
-        <v/>
-      </c>
-      <c r="AM13" s="24">
-        <f>AG13+AH13+AI13+AL13</f>
-        <v/>
-      </c>
-      <c r="AN13" s="25">
-        <f>IF(AM13&gt;0, AG13/AM13, 0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="26" t="inlineStr">
-        <is>
-          <t>MANI
-Employee</t>
-        </is>
-      </c>
-      <c r="B14" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="C14" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="D14" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="E14" s="15" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="F14" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="G14" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="H14" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="I14" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="J14" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="K14" s="27" t="inlineStr">
-        <is>
-          <t>CF</t>
-        </is>
-      </c>
-      <c r="L14" s="16" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="M14" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="N14" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="O14" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="P14" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q14" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="R14" s="16" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="S14" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="T14" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="U14" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="V14" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="W14" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="X14" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="X14" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
         </is>
       </c>
       <c r="Y14" s="13" t="inlineStr">
@@ -2957,19 +2957,19 @@
           <t>P</t>
         </is>
       </c>
-      <c r="AA14" s="16" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="AB14" s="16" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="AC14" s="16" t="inlineStr">
-        <is>
-          <t>L</t>
+      <c r="AA14" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AB14" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AC14" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
         </is>
       </c>
       <c r="AD14" s="13" t="inlineStr">
@@ -2982,40 +2982,40 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="AF14" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG14" s="18">
+      <c r="AF14" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG14" s="16">
         <f>COUNTIF(B14:AF14, "P")</f>
         <v/>
       </c>
-      <c r="AH14" s="19">
+      <c r="AH14" s="17">
         <f>COUNTIF(B14:AF14, "CL")</f>
         <v/>
       </c>
-      <c r="AI14" s="20">
+      <c r="AI14" s="18">
         <f>COUNTIF(B14:AF14, "L")</f>
         <v/>
       </c>
-      <c r="AJ14" s="21">
+      <c r="AJ14" s="19">
         <f>COUNTIF(B14:AF14, "WO")</f>
         <v/>
       </c>
-      <c r="AK14" s="22">
+      <c r="AK14" s="20">
         <f>COUNTIF(B14:AF14, "HO")</f>
         <v/>
       </c>
-      <c r="AL14" s="23">
+      <c r="AL14" s="21">
         <f>COUNTIF(B14:AF14, "CF")</f>
         <v/>
       </c>
-      <c r="AM14" s="24">
+      <c r="AM14" s="22">
         <f>AG14+AH14+AI14+AL14</f>
         <v/>
       </c>
-      <c r="AN14" s="25">
+      <c r="AN14" s="23">
         <f>IF(AM14&gt;0, AG14/AM14, 0)</f>
         <v/>
       </c>
@@ -3023,7 +3023,7 @@
     <row r="15" ht="32" customHeight="1">
       <c r="A15" s="12" t="inlineStr">
         <is>
-          <t>NEELIMA
+          <t>VANI
 Employee</t>
         </is>
       </c>
@@ -3052,9 +3052,9 @@
           <t>P</t>
         </is>
       </c>
-      <c r="G15" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="G15" s="25" t="inlineStr">
+        <is>
+          <t>CL</t>
         </is>
       </c>
       <c r="H15" s="13" t="inlineStr">
@@ -3097,14 +3097,14 @@
           <t>P</t>
         </is>
       </c>
-      <c r="P15" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="Q15" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="P15" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q15" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
         </is>
       </c>
       <c r="R15" s="13" t="inlineStr">
@@ -3177,48 +3177,48 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="AF15" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG15" s="18">
+      <c r="AF15" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG15" s="16">
         <f>COUNTIF(B15:AF15, "P")</f>
         <v/>
       </c>
-      <c r="AH15" s="19">
+      <c r="AH15" s="17">
         <f>COUNTIF(B15:AF15, "CL")</f>
         <v/>
       </c>
-      <c r="AI15" s="20">
+      <c r="AI15" s="18">
         <f>COUNTIF(B15:AF15, "L")</f>
         <v/>
       </c>
-      <c r="AJ15" s="21">
+      <c r="AJ15" s="19">
         <f>COUNTIF(B15:AF15, "WO")</f>
         <v/>
       </c>
-      <c r="AK15" s="22">
+      <c r="AK15" s="20">
         <f>COUNTIF(B15:AF15, "HO")</f>
         <v/>
       </c>
-      <c r="AL15" s="23">
+      <c r="AL15" s="21">
         <f>COUNTIF(B15:AF15, "CF")</f>
         <v/>
       </c>
-      <c r="AM15" s="24">
+      <c r="AM15" s="22">
         <f>AG15+AH15+AI15+AL15</f>
         <v/>
       </c>
-      <c r="AN15" s="25">
+      <c r="AN15" s="23">
         <f>IF(AM15&gt;0, AG15/AM15, 0)</f>
         <v/>
       </c>
     </row>
     <row r="16" ht="32" customHeight="1">
-      <c r="A16" s="26" t="inlineStr">
-        <is>
-          <t>PHANI
+      <c r="A16" s="24" t="inlineStr">
+        <is>
+          <t>Ch Praveen Kumar
 Employee</t>
         </is>
       </c>
@@ -3247,29 +3247,29 @@
           <t>P</t>
         </is>
       </c>
-      <c r="G16" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="H16" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="I16" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="J16" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="K16" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
+      <c r="G16" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="H16" s="25" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="I16" s="27" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="J16" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="K16" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
         </is>
       </c>
       <c r="L16" s="13" t="inlineStr">
@@ -3292,14 +3292,14 @@
           <t>P</t>
         </is>
       </c>
-      <c r="P16" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q16" s="15" t="inlineStr">
-        <is>
-          <t>CL</t>
+      <c r="P16" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Q16" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
         </is>
       </c>
       <c r="R16" s="13" t="inlineStr">
@@ -3322,90 +3322,90 @@
           <t>P</t>
         </is>
       </c>
-      <c r="V16" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="W16" s="27" t="inlineStr">
-        <is>
-          <t>CF</t>
-        </is>
-      </c>
-      <c r="X16" s="27" t="inlineStr">
-        <is>
-          <t>CF</t>
-        </is>
-      </c>
-      <c r="Y16" s="27" t="inlineStr">
-        <is>
-          <t>CF</t>
-        </is>
-      </c>
-      <c r="Z16" s="27" t="inlineStr">
-        <is>
-          <t>CF</t>
-        </is>
-      </c>
-      <c r="AA16" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="AB16" s="16" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="AC16" s="16" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="AD16" s="16" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="AE16" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AF16" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG16" s="18">
+      <c r="V16" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="W16" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="X16" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="Y16" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Z16" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AA16" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AB16" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AC16" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AD16" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AE16" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="AF16" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG16" s="16">
         <f>COUNTIF(B16:AF16, "P")</f>
         <v/>
       </c>
-      <c r="AH16" s="19">
+      <c r="AH16" s="17">
         <f>COUNTIF(B16:AF16, "CL")</f>
         <v/>
       </c>
-      <c r="AI16" s="20">
+      <c r="AI16" s="18">
         <f>COUNTIF(B16:AF16, "L")</f>
         <v/>
       </c>
-      <c r="AJ16" s="21">
+      <c r="AJ16" s="19">
         <f>COUNTIF(B16:AF16, "WO")</f>
         <v/>
       </c>
-      <c r="AK16" s="22">
+      <c r="AK16" s="20">
         <f>COUNTIF(B16:AF16, "HO")</f>
         <v/>
       </c>
-      <c r="AL16" s="23">
+      <c r="AL16" s="21">
         <f>COUNTIF(B16:AF16, "CF")</f>
         <v/>
       </c>
-      <c r="AM16" s="24">
+      <c r="AM16" s="22">
         <f>AG16+AH16+AI16+AL16</f>
         <v/>
       </c>
-      <c r="AN16" s="25">
+      <c r="AN16" s="23">
         <f>IF(AM16&gt;0, AG16/AM16, 0)</f>
         <v/>
       </c>
@@ -3413,202 +3413,202 @@
     <row r="17" ht="32" customHeight="1">
       <c r="A17" s="12" t="inlineStr">
         <is>
-          <t>PRAVEEN KUMAR
+          <t>KAVITHA
 Employee</t>
         </is>
       </c>
-      <c r="B17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="U17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Z17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AA17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AC17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AD17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AE17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AF17" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG17" s="18">
+      <c r="B17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C17" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="D17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="E17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="F17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="G17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="H17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="I17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="J17" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="K17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="L17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="M17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="N17" s="25" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="O17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="P17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Q17" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="R17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="S17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="T17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="U17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="V17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="W17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="X17" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="Y17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Z17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AA17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AB17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AC17" s="27" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="AD17" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AE17" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="AF17" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG17" s="16">
         <f>COUNTIF(B17:AF17, "P")</f>
         <v/>
       </c>
-      <c r="AH17" s="19">
+      <c r="AH17" s="17">
         <f>COUNTIF(B17:AF17, "CL")</f>
         <v/>
       </c>
-      <c r="AI17" s="20">
+      <c r="AI17" s="18">
         <f>COUNTIF(B17:AF17, "L")</f>
         <v/>
       </c>
-      <c r="AJ17" s="21">
+      <c r="AJ17" s="19">
         <f>COUNTIF(B17:AF17, "WO")</f>
         <v/>
       </c>
-      <c r="AK17" s="22">
+      <c r="AK17" s="20">
         <f>COUNTIF(B17:AF17, "HO")</f>
         <v/>
       </c>
-      <c r="AL17" s="23">
+      <c r="AL17" s="21">
         <f>COUNTIF(B17:AF17, "CF")</f>
         <v/>
       </c>
-      <c r="AM17" s="24">
+      <c r="AM17" s="22">
         <f>AG17+AH17+AI17+AL17</f>
         <v/>
       </c>
-      <c r="AN17" s="25">
+      <c r="AN17" s="23">
         <f>IF(AM17&gt;0, AG17/AM17, 0)</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="32" customHeight="1">
-      <c r="A18" s="26" t="inlineStr">
-        <is>
-          <t>RAMESH
+      <c r="A18" s="24" t="inlineStr">
+        <is>
+          <t>VAIDEHI
 Employee</t>
         </is>
       </c>
@@ -3647,9 +3647,9 @@
           <t>P</t>
         </is>
       </c>
-      <c r="I18" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="I18" s="25" t="inlineStr">
+        <is>
+          <t>CL</t>
         </is>
       </c>
       <c r="J18" s="14" t="inlineStr">
@@ -3657,9 +3657,9 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="K18" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="K18" s="26" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="L18" s="13" t="inlineStr">
@@ -3682,7 +3682,7 @@
           <t>P</t>
         </is>
       </c>
-      <c r="P18" s="17" t="inlineStr">
+      <c r="P18" s="15" t="inlineStr">
         <is>
           <t>-</t>
         </is>
@@ -3762,40 +3762,40 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="AF18" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG18" s="18">
+      <c r="AF18" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG18" s="16">
         <f>COUNTIF(B18:AF18, "P")</f>
         <v/>
       </c>
-      <c r="AH18" s="19">
+      <c r="AH18" s="17">
         <f>COUNTIF(B18:AF18, "CL")</f>
         <v/>
       </c>
-      <c r="AI18" s="20">
+      <c r="AI18" s="18">
         <f>COUNTIF(B18:AF18, "L")</f>
         <v/>
       </c>
-      <c r="AJ18" s="21">
+      <c r="AJ18" s="19">
         <f>COUNTIF(B18:AF18, "WO")</f>
         <v/>
       </c>
-      <c r="AK18" s="22">
+      <c r="AK18" s="20">
         <f>COUNTIF(B18:AF18, "HO")</f>
         <v/>
       </c>
-      <c r="AL18" s="23">
+      <c r="AL18" s="21">
         <f>COUNTIF(B18:AF18, "CF")</f>
         <v/>
       </c>
-      <c r="AM18" s="24">
+      <c r="AM18" s="22">
         <f>AG18+AH18+AI18+AL18</f>
         <v/>
       </c>
-      <c r="AN18" s="25">
+      <c r="AN18" s="23">
         <f>IF(AM18&gt;0, AG18/AM18, 0)</f>
         <v/>
       </c>
@@ -3803,202 +3803,202 @@
     <row r="19" ht="32" customHeight="1">
       <c r="A19" s="12" t="inlineStr">
         <is>
-          <t>RAVALI
+          <t>VAISHNAVI
 Employee</t>
         </is>
       </c>
-      <c r="B19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="U19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Z19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AA19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AC19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AD19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AE19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AF19" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG19" s="18">
+      <c r="B19" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="C19" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="D19" s="25" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="E19" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="F19" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="G19" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="H19" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="I19" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="J19" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="K19" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="L19" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="M19" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="N19" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="O19" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="P19" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q19" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="R19" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="S19" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="T19" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="U19" s="26" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="V19" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="W19" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="X19" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="Y19" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="Z19" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AA19" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AB19" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AC19" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AD19" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AE19" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="AF19" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG19" s="16">
         <f>COUNTIF(B19:AF19, "P")</f>
         <v/>
       </c>
-      <c r="AH19" s="19">
+      <c r="AH19" s="17">
         <f>COUNTIF(B19:AF19, "CL")</f>
         <v/>
       </c>
-      <c r="AI19" s="20">
+      <c r="AI19" s="18">
         <f>COUNTIF(B19:AF19, "L")</f>
         <v/>
       </c>
-      <c r="AJ19" s="21">
+      <c r="AJ19" s="19">
         <f>COUNTIF(B19:AF19, "WO")</f>
         <v/>
       </c>
-      <c r="AK19" s="22">
+      <c r="AK19" s="20">
         <f>COUNTIF(B19:AF19, "HO")</f>
         <v/>
       </c>
-      <c r="AL19" s="23">
+      <c r="AL19" s="21">
         <f>COUNTIF(B19:AF19, "CF")</f>
         <v/>
       </c>
-      <c r="AM19" s="24">
+      <c r="AM19" s="22">
         <f>AG19+AH19+AI19+AL19</f>
         <v/>
       </c>
-      <c r="AN19" s="25">
+      <c r="AN19" s="23">
         <f>IF(AM19&gt;0, AG19/AM19, 0)</f>
         <v/>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
-      <c r="A20" s="26" t="inlineStr">
-        <is>
-          <t>SAI CHARAN
+      <c r="A20" s="24" t="inlineStr">
+        <is>
+          <t>SIRISHA
 Employee</t>
         </is>
       </c>
@@ -4017,9 +4017,9 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E20" s="16" t="inlineStr">
-        <is>
-          <t>L</t>
+      <c r="E20" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
         </is>
       </c>
       <c r="F20" s="13" t="inlineStr">
@@ -4072,9 +4072,9 @@
           <t>P</t>
         </is>
       </c>
-      <c r="P20" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
+      <c r="P20" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
         </is>
       </c>
       <c r="Q20" s="14" t="inlineStr">
@@ -4102,14 +4102,14 @@
           <t>P</t>
         </is>
       </c>
-      <c r="V20" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="W20" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="V20" s="25" t="inlineStr">
+        <is>
+          <t>CL</t>
+        </is>
+      </c>
+      <c r="W20" s="27" t="inlineStr">
+        <is>
+          <t>CF</t>
         </is>
       </c>
       <c r="X20" s="14" t="inlineStr">
@@ -4122,9 +4122,9 @@
           <t>P</t>
         </is>
       </c>
-      <c r="Z20" s="16" t="inlineStr">
-        <is>
-          <t>L</t>
+      <c r="Z20" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
         </is>
       </c>
       <c r="AA20" s="13" t="inlineStr">
@@ -4137,14 +4137,14 @@
           <t>P</t>
         </is>
       </c>
-      <c r="AC20" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AD20" s="16" t="inlineStr">
-        <is>
-          <t>L</t>
+      <c r="AC20" s="27" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="AD20" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
         </is>
       </c>
       <c r="AE20" s="14" t="inlineStr">
@@ -4152,40 +4152,40 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="AF20" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG20" s="18">
+      <c r="AF20" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG20" s="16">
         <f>COUNTIF(B20:AF20, "P")</f>
         <v/>
       </c>
-      <c r="AH20" s="19">
+      <c r="AH20" s="17">
         <f>COUNTIF(B20:AF20, "CL")</f>
         <v/>
       </c>
-      <c r="AI20" s="20">
+      <c r="AI20" s="18">
         <f>COUNTIF(B20:AF20, "L")</f>
         <v/>
       </c>
-      <c r="AJ20" s="21">
+      <c r="AJ20" s="19">
         <f>COUNTIF(B20:AF20, "WO")</f>
         <v/>
       </c>
-      <c r="AK20" s="22">
+      <c r="AK20" s="20">
         <f>COUNTIF(B20:AF20, "HO")</f>
         <v/>
       </c>
-      <c r="AL20" s="23">
+      <c r="AL20" s="21">
         <f>COUNTIF(B20:AF20, "CF")</f>
         <v/>
       </c>
-      <c r="AM20" s="24">
+      <c r="AM20" s="22">
         <f>AG20+AH20+AI20+AL20</f>
         <v/>
       </c>
-      <c r="AN20" s="25">
+      <c r="AN20" s="23">
         <f>IF(AM20&gt;0, AG20/AM20, 0)</f>
         <v/>
       </c>
@@ -4193,7 +4193,7 @@
     <row r="21" ht="32" customHeight="1">
       <c r="A21" s="12" t="inlineStr">
         <is>
-          <t>SAI KUMAR
+          <t>SAI CHARAN
 Employee</t>
         </is>
       </c>
@@ -4212,9 +4212,9 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E21" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="E21" s="26" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="F21" s="13" t="inlineStr">
@@ -4237,9 +4237,9 @@
           <t>P</t>
         </is>
       </c>
-      <c r="J21" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="J21" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
         </is>
       </c>
       <c r="K21" s="13" t="inlineStr">
@@ -4267,9 +4267,9 @@
           <t>P</t>
         </is>
       </c>
-      <c r="P21" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="P21" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="Q21" s="14" t="inlineStr">
@@ -4317,9 +4317,9 @@
           <t>P</t>
         </is>
       </c>
-      <c r="Z21" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="Z21" s="26" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="AA21" s="13" t="inlineStr">
@@ -4332,14 +4332,14 @@
           <t>P</t>
         </is>
       </c>
-      <c r="AC21" s="15" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="AD21" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="AC21" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AD21" s="26" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="AE21" s="14" t="inlineStr">
@@ -4347,48 +4347,48 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="AF21" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG21" s="18">
+      <c r="AF21" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG21" s="16">
         <f>COUNTIF(B21:AF21, "P")</f>
         <v/>
       </c>
-      <c r="AH21" s="19">
+      <c r="AH21" s="17">
         <f>COUNTIF(B21:AF21, "CL")</f>
         <v/>
       </c>
-      <c r="AI21" s="20">
+      <c r="AI21" s="18">
         <f>COUNTIF(B21:AF21, "L")</f>
         <v/>
       </c>
-      <c r="AJ21" s="21">
+      <c r="AJ21" s="19">
         <f>COUNTIF(B21:AF21, "WO")</f>
         <v/>
       </c>
-      <c r="AK21" s="22">
+      <c r="AK21" s="20">
         <f>COUNTIF(B21:AF21, "HO")</f>
         <v/>
       </c>
-      <c r="AL21" s="23">
+      <c r="AL21" s="21">
         <f>COUNTIF(B21:AF21, "CF")</f>
         <v/>
       </c>
-      <c r="AM21" s="24">
+      <c r="AM21" s="22">
         <f>AG21+AH21+AI21+AL21</f>
         <v/>
       </c>
-      <c r="AN21" s="25">
+      <c r="AN21" s="23">
         <f>IF(AM21&gt;0, AG21/AM21, 0)</f>
         <v/>
       </c>
     </row>
     <row r="22" ht="32" customHeight="1">
-      <c r="A22" s="26" t="inlineStr">
-        <is>
-          <t>SIRISHA
+      <c r="A22" s="24" t="inlineStr">
+        <is>
+          <t>MANI
 Employee</t>
         </is>
       </c>
@@ -4407,9 +4407,9 @@
           <t>P</t>
         </is>
       </c>
-      <c r="E22" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="E22" s="25" t="inlineStr">
+        <is>
+          <t>CL</t>
         </is>
       </c>
       <c r="F22" s="13" t="inlineStr">
@@ -4437,14 +4437,14 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="K22" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="L22" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="K22" s="27" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="L22" s="26" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="M22" s="13" t="inlineStr">
@@ -4462,9 +4462,9 @@
           <t>P</t>
         </is>
       </c>
-      <c r="P22" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="P22" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="Q22" s="14" t="inlineStr">
@@ -4472,9 +4472,9 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="R22" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="R22" s="26" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="S22" s="13" t="inlineStr">
@@ -4492,19 +4492,19 @@
           <t>P</t>
         </is>
       </c>
-      <c r="V22" s="15" t="inlineStr">
-        <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="W22" s="27" t="inlineStr">
-        <is>
-          <t>CF</t>
-        </is>
-      </c>
-      <c r="X22" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
+      <c r="V22" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="W22" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="X22" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
         </is>
       </c>
       <c r="Y22" s="13" t="inlineStr">
@@ -4517,19 +4517,19 @@
           <t>P</t>
         </is>
       </c>
-      <c r="AA22" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AB22" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AC22" s="27" t="inlineStr">
-        <is>
-          <t>CF</t>
+      <c r="AA22" s="26" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="AB22" s="26" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="AC22" s="26" t="inlineStr">
+        <is>
+          <t>L</t>
         </is>
       </c>
       <c r="AD22" s="13" t="inlineStr">
@@ -4542,40 +4542,40 @@
           <t>WO</t>
         </is>
       </c>
-      <c r="AF22" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG22" s="18">
+      <c r="AF22" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG22" s="16">
         <f>COUNTIF(B22:AF22, "P")</f>
         <v/>
       </c>
-      <c r="AH22" s="19">
+      <c r="AH22" s="17">
         <f>COUNTIF(B22:AF22, "CL")</f>
         <v/>
       </c>
-      <c r="AI22" s="20">
+      <c r="AI22" s="18">
         <f>COUNTIF(B22:AF22, "L")</f>
         <v/>
       </c>
-      <c r="AJ22" s="21">
+      <c r="AJ22" s="19">
         <f>COUNTIF(B22:AF22, "WO")</f>
         <v/>
       </c>
-      <c r="AK22" s="22">
+      <c r="AK22" s="20">
         <f>COUNTIF(B22:AF22, "HO")</f>
         <v/>
       </c>
-      <c r="AL22" s="23">
+      <c r="AL22" s="21">
         <f>COUNTIF(B22:AF22, "CF")</f>
         <v/>
       </c>
-      <c r="AM22" s="24">
+      <c r="AM22" s="22">
         <f>AG22+AH22+AI22+AL22</f>
         <v/>
       </c>
-      <c r="AN22" s="25">
+      <c r="AN22" s="23">
         <f>IF(AM22&gt;0, AG22/AM22, 0)</f>
         <v/>
       </c>
@@ -4583,7 +4583,7 @@
     <row r="23" ht="32" customHeight="1">
       <c r="A23" s="12" t="inlineStr">
         <is>
-          <t>VAIDEHI
+          <t>PHANI
 Employee</t>
         </is>
       </c>
@@ -4592,9 +4592,9 @@
           <t>P</t>
         </is>
       </c>
-      <c r="C23" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
+      <c r="C23" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
         </is>
       </c>
       <c r="D23" s="13" t="inlineStr">
@@ -4612,9 +4612,9 @@
           <t>P</t>
         </is>
       </c>
-      <c r="G23" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="G23" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
         </is>
       </c>
       <c r="H23" s="13" t="inlineStr">
@@ -4622,350 +4622,350 @@
           <t>P</t>
         </is>
       </c>
-      <c r="I23" s="15" t="inlineStr">
+      <c r="I23" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="J23" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="K23" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="L23" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="M23" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="N23" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="O23" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="P23" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q23" s="25" t="inlineStr">
         <is>
           <t>CL</t>
         </is>
       </c>
-      <c r="J23" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="K23" s="16" t="inlineStr">
+      <c r="R23" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="S23" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="T23" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="U23" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="V23" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="W23" s="27" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="X23" s="27" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="Y23" s="27" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="Z23" s="27" t="inlineStr">
+        <is>
+          <t>CF</t>
+        </is>
+      </c>
+      <c r="AA23" s="14" t="inlineStr">
+        <is>
+          <t>WO</t>
+        </is>
+      </c>
+      <c r="AB23" s="26" t="inlineStr">
         <is>
           <t>L</t>
         </is>
       </c>
-      <c r="L23" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="M23" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="N23" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="O23" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="P23" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q23" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="R23" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="S23" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="T23" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="U23" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="V23" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="W23" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="X23" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="Y23" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="Z23" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AA23" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AB23" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AC23" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AD23" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AE23" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="AF23" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG23" s="18">
+      <c r="AC23" s="26" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="AD23" s="26" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="AE23" s="13" t="inlineStr">
+        <is>
+          <t>P</t>
+        </is>
+      </c>
+      <c r="AF23" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG23" s="16">
         <f>COUNTIF(B23:AF23, "P")</f>
         <v/>
       </c>
-      <c r="AH23" s="19">
+      <c r="AH23" s="17">
         <f>COUNTIF(B23:AF23, "CL")</f>
         <v/>
       </c>
-      <c r="AI23" s="20">
+      <c r="AI23" s="18">
         <f>COUNTIF(B23:AF23, "L")</f>
         <v/>
       </c>
-      <c r="AJ23" s="21">
+      <c r="AJ23" s="19">
         <f>COUNTIF(B23:AF23, "WO")</f>
         <v/>
       </c>
-      <c r="AK23" s="22">
+      <c r="AK23" s="20">
         <f>COUNTIF(B23:AF23, "HO")</f>
         <v/>
       </c>
-      <c r="AL23" s="23">
+      <c r="AL23" s="21">
         <f>COUNTIF(B23:AF23, "CF")</f>
         <v/>
       </c>
-      <c r="AM23" s="24">
+      <c r="AM23" s="22">
         <f>AG23+AH23+AI23+AL23</f>
         <v/>
       </c>
-      <c r="AN23" s="25">
+      <c r="AN23" s="23">
         <f>IF(AM23&gt;0, AG23/AM23, 0)</f>
         <v/>
       </c>
     </row>
     <row r="24" ht="32" customHeight="1">
-      <c r="A24" s="26" t="inlineStr">
-        <is>
-          <t>VAISHNAVI
+      <c r="A24" s="24" t="inlineStr">
+        <is>
+          <t>PRAVEEN KUMAR
 Employee</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="C24" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
+      <c r="B24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="D24" s="15" t="inlineStr">
         <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="E24" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="F24" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="G24" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="H24" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="I24" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="J24" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="K24" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="L24" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="M24" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="N24" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="O24" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="P24" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q24" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="R24" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="S24" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="T24" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="U24" s="16" t="inlineStr">
-        <is>
-          <t>L</t>
-        </is>
-      </c>
-      <c r="V24" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="W24" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="X24" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="Y24" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="Z24" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AA24" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AB24" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AC24" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AD24" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AE24" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="AF24" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG24" s="18">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AD24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF24" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG24" s="16">
         <f>COUNTIF(B24:AF24, "P")</f>
         <v/>
       </c>
-      <c r="AH24" s="19">
+      <c r="AH24" s="17">
         <f>COUNTIF(B24:AF24, "CL")</f>
         <v/>
       </c>
-      <c r="AI24" s="20">
+      <c r="AI24" s="18">
         <f>COUNTIF(B24:AF24, "L")</f>
         <v/>
       </c>
-      <c r="AJ24" s="21">
+      <c r="AJ24" s="19">
         <f>COUNTIF(B24:AF24, "WO")</f>
         <v/>
       </c>
-      <c r="AK24" s="22">
+      <c r="AK24" s="20">
         <f>COUNTIF(B24:AF24, "HO")</f>
         <v/>
       </c>
-      <c r="AL24" s="23">
+      <c r="AL24" s="21">
         <f>COUNTIF(B24:AF24, "CF")</f>
         <v/>
       </c>
-      <c r="AM24" s="24">
+      <c r="AM24" s="22">
         <f>AG24+AH24+AI24+AL24</f>
         <v/>
       </c>
-      <c r="AN24" s="25">
+      <c r="AN24" s="23">
         <f>IF(AM24&gt;0, AG24/AM24, 0)</f>
         <v/>
       </c>
@@ -4973,389 +4973,389 @@
     <row r="25" ht="32" customHeight="1">
       <c r="A25" s="12" t="inlineStr">
         <is>
-          <t>VANI
+          <t>RAVALI
 Employee</t>
         </is>
       </c>
-      <c r="B25" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="C25" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="D25" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="E25" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="F25" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
+      <c r="B25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
         </is>
       </c>
       <c r="G25" s="15" t="inlineStr">
         <is>
-          <t>CL</t>
-        </is>
-      </c>
-      <c r="H25" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="I25" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="J25" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="K25" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="L25" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="M25" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="N25" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="O25" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="P25" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q25" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="R25" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="S25" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="T25" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="U25" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="V25" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="W25" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="X25" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="Y25" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="Z25" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AA25" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AB25" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AC25" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AD25" s="13" t="inlineStr">
-        <is>
-          <t>P</t>
-        </is>
-      </c>
-      <c r="AE25" s="14" t="inlineStr">
-        <is>
-          <t>WO</t>
-        </is>
-      </c>
-      <c r="AF25" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG25" s="18">
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AD25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF25" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG25" s="16">
         <f>COUNTIF(B25:AF25, "P")</f>
         <v/>
       </c>
-      <c r="AH25" s="19">
+      <c r="AH25" s="17">
         <f>COUNTIF(B25:AF25, "CL")</f>
         <v/>
       </c>
-      <c r="AI25" s="20">
+      <c r="AI25" s="18">
         <f>COUNTIF(B25:AF25, "L")</f>
         <v/>
       </c>
-      <c r="AJ25" s="21">
+      <c r="AJ25" s="19">
         <f>COUNTIF(B25:AF25, "WO")</f>
         <v/>
       </c>
-      <c r="AK25" s="22">
+      <c r="AK25" s="20">
         <f>COUNTIF(B25:AF25, "HO")</f>
         <v/>
       </c>
-      <c r="AL25" s="23">
+      <c r="AL25" s="21">
         <f>COUNTIF(B25:AF25, "CF")</f>
         <v/>
       </c>
-      <c r="AM25" s="24">
+      <c r="AM25" s="22">
         <f>AG25+AH25+AI25+AL25</f>
         <v/>
       </c>
-      <c r="AN25" s="25">
+      <c r="AN25" s="23">
         <f>IF(AM25&gt;0, AG25/AM25, 0)</f>
         <v/>
       </c>
     </row>
     <row r="26" ht="32" customHeight="1">
-      <c r="A26" s="26" t="inlineStr">
+      <c r="A26" s="24" t="inlineStr">
         <is>
           <t>VITTAL
 Employee</t>
         </is>
       </c>
-      <c r="B26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="C26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="F26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="G26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="H26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="J26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="L26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="M26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="N26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="O26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="P26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Q26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="R26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="S26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="T26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="U26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="V26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="W26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="X26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Y26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="Z26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AA26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AB26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AC26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AD26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AE26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AF26" s="17" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AG26" s="18">
+      <c r="B26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="I26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="J26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="L26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="M26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="N26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="O26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="P26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Q26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="R26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="S26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="T26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="U26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="V26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="W26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="X26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Y26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="Z26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AA26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AB26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AC26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AD26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AE26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AF26" s="15" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AG26" s="16">
         <f>COUNTIF(B26:AF26, "P")</f>
         <v/>
       </c>
-      <c r="AH26" s="19">
+      <c r="AH26" s="17">
         <f>COUNTIF(B26:AF26, "CL")</f>
         <v/>
       </c>
-      <c r="AI26" s="20">
+      <c r="AI26" s="18">
         <f>COUNTIF(B26:AF26, "L")</f>
         <v/>
       </c>
-      <c r="AJ26" s="21">
+      <c r="AJ26" s="19">
         <f>COUNTIF(B26:AF26, "WO")</f>
         <v/>
       </c>
-      <c r="AK26" s="22">
+      <c r="AK26" s="20">
         <f>COUNTIF(B26:AF26, "HO")</f>
         <v/>
       </c>
-      <c r="AL26" s="23">
+      <c r="AL26" s="21">
         <f>COUNTIF(B26:AF26, "CF")</f>
         <v/>
       </c>
-      <c r="AM26" s="24">
+      <c r="AM26" s="22">
         <f>AG26+AH26+AI26+AL26</f>
         <v/>
       </c>
-      <c r="AN26" s="25">
+      <c r="AN26" s="23">
         <f>IF(AM26&gt;0, AG26/AM26, 0)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Remove 'ranked in descending order' banner text while preserving sorted order
</commit_message>
<xml_diff>
--- a/Vasus_Attendance_August_2026.xlsx
+++ b/Vasus_Attendance_August_2026.xlsx
@@ -823,14 +823,14 @@
     <row r="1" ht="36" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>VASUS ATTENDANCE TRACKER — AUGUST 2026 (RANKED IN DESCENDING ORDER)</t>
+          <t>VASUS ATTENDANCE TRACKER — AUGUST 2026</t>
         </is>
       </c>
     </row>
     <row r="2" ht="24" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Doctors &amp; Employees ranked in descending order separately  |  [P] Present (Green)  [CL] Casual Leave (Teal)  [L] Leave (Red)  [WO] Week Off (Purple)  [CF] Comp Off (Pink)</t>
+          <t>Status Codes:  [P] Present (Green)  |  [CL] Casual Leave (Teal)  |  [L] Leave (Red)  |  [WO] Week Off (Purple)  |  [HO] Holiday (Mint)  |  [CF] Comp Off (Pink)  |  [-] Blank</t>
         </is>
       </c>
     </row>

</xml_diff>